<commit_message>
Call list: row heights
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/CALL_LIST_1510.xlsx
+++ b/CALL_LIST_1510.xlsx
@@ -627,7 +627,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="272" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
@@ -712,7 +712,7 @@
       <c r="N4" s="6" t="inlineStr"/>
       <c r="O4" s="6" t="inlineStr"/>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="272" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
@@ -795,7 +795,7 @@
       <c r="N5" s="6" t="inlineStr"/>
       <c r="O5" s="6" t="inlineStr"/>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="253" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -876,7 +876,7 @@
       <c r="N6" s="6" t="inlineStr"/>
       <c r="O6" s="6" t="inlineStr"/>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="177" customHeight="1">
       <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
@@ -950,7 +950,7 @@
       <c r="N7" s="6" t="inlineStr"/>
       <c r="O7" s="6" t="inlineStr"/>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="215" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
@@ -1029,7 +1029,7 @@
       <c r="N8" s="6" t="inlineStr"/>
       <c r="O8" s="6" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="63" customHeight="1">
       <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
@@ -1092,7 +1092,7 @@
       <c r="N9" s="6" t="inlineStr"/>
       <c r="O9" s="6" t="inlineStr"/>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
@@ -1152,7 +1152,7 @@
       <c r="N10" s="6" t="inlineStr"/>
       <c r="O10" s="6" t="inlineStr"/>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
@@ -1207,7 +1207,7 @@
       <c r="N11" s="6" t="inlineStr"/>
       <c r="O11" s="6" t="inlineStr"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="63" customHeight="1">
       <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
@@ -1270,7 +1270,7 @@
       <c r="N12" s="6" t="inlineStr"/>
       <c r="O12" s="6" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
@@ -1329,7 +1329,7 @@
       <c r="N13" s="6" t="inlineStr"/>
       <c r="O13" s="6" t="inlineStr"/>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="n">
         <v>11</v>
       </c>
@@ -1388,7 +1388,7 @@
       <c r="N14" s="6" t="inlineStr"/>
       <c r="O14" s="6" t="inlineStr"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
         <v>12</v>
       </c>
@@ -1447,7 +1447,7 @@
       <c r="N15" s="6" t="inlineStr"/>
       <c r="O15" s="6" t="inlineStr"/>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="30" customHeight="1">
       <c r="A16" s="4" t="n">
         <v>13</v>
       </c>
@@ -1506,7 +1506,7 @@
       <c r="N16" s="6" t="inlineStr"/>
       <c r="O16" s="6" t="inlineStr"/>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
         <v>14</v>
       </c>
@@ -1565,7 +1565,7 @@
       <c r="N17" s="6" t="inlineStr"/>
       <c r="O17" s="6" t="inlineStr"/>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="44" customHeight="1">
       <c r="A18" s="4" t="n">
         <v>15</v>
       </c>
@@ -1625,7 +1625,7 @@
       <c r="N18" s="6" t="inlineStr"/>
       <c r="O18" s="6" t="inlineStr"/>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
         <v>16</v>
       </c>
@@ -1684,7 +1684,7 @@
       <c r="N19" s="6" t="inlineStr"/>
       <c r="O19" s="6" t="inlineStr"/>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20" ht="30" customHeight="1">
       <c r="A20" s="4" t="n">
         <v>17</v>
       </c>
@@ -1743,7 +1743,7 @@
       <c r="N20" s="6" t="inlineStr"/>
       <c r="O20" s="6" t="inlineStr"/>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
         <v>18</v>
       </c>
@@ -1802,7 +1802,7 @@
       <c r="N21" s="6" t="inlineStr"/>
       <c r="O21" s="6" t="inlineStr"/>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="30" customHeight="1">
       <c r="A22" s="4" t="n">
         <v>19</v>
       </c>
@@ -1861,7 +1861,7 @@
       <c r="N22" s="6" t="inlineStr"/>
       <c r="O22" s="6" t="inlineStr"/>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
         <v>20</v>
       </c>
@@ -1916,7 +1916,7 @@
       <c r="N23" s="6" t="inlineStr"/>
       <c r="O23" s="6" t="inlineStr"/>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24" ht="30" customHeight="1">
       <c r="A24" s="4" t="n">
         <v>21</v>
       </c>

</xml_diff>